<commit_message>
Lock all 6 templates: workbook structure protected, all cells locked, sheets protected. Prevents modification of content, formulas, and structure.
</commit_message>
<xml_diff>
--- a/downloads/free-resources/ahqs-audit-tool-template.xlsx
+++ b/downloads/free-resources/ahqs-audit-tool-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
+  <workbookProtection workbookPassword="AF18" lockStructure="1" lockWindows="0"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
@@ -634,7 +634,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
               </a:p>
             </txPr>
@@ -797,7 +797,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -887,7 +887,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -920,7 +920,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
         </a:p>
       </txPr>
@@ -1085,7 +1085,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                 </a:p>
               </txPr>
@@ -1113,7 +1113,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                 </a:p>
               </txPr>
@@ -1141,7 +1141,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                 </a:p>
               </txPr>
@@ -1169,7 +1169,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                 </a:p>
               </txPr>
@@ -1197,7 +1197,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                 </a:p>
               </txPr>
@@ -1223,7 +1223,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
               </a:p>
             </txPr>
@@ -1310,7 +1310,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
         </a:p>
       </txPr>
@@ -1619,7 +1619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B9:C34"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="23" min="1" max="1"/>
@@ -1627,6 +1627,14 @@
     <col width="3" customWidth="1" style="23" min="3" max="3"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
     <row r="9" ht="26.25" customHeight="1" s="24">
       <c r="B9" s="25" t="inlineStr">
         <is>
@@ -1641,6 +1649,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="15" customHeight="1" s="24">
       <c r="B12" s="27" t="n"/>
       <c r="C12" s="27" t="n"/>
@@ -1652,6 +1661,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="15.75" customHeight="1" s="24">
       <c r="B15" s="29" t="inlineStr">
         <is>
@@ -1701,6 +1711,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="15.75" customHeight="1" s="24">
       <c r="B23" s="29" t="inlineStr">
         <is>
@@ -1750,6 +1761,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31" ht="15.75" customHeight="1" s="24">
       <c r="B31" s="29" t="inlineStr">
         <is>
@@ -1764,6 +1776,7 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34" ht="15" customHeight="1" s="24">
       <c r="B34" s="32" t="inlineStr">
         <is>
@@ -1772,6 +1785,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="AF18"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1969,6 +1983,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="AF18"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3096,6 +3111,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="AF18"/>
   <autoFilter ref="A1:M51"/>
   <conditionalFormatting sqref="E2:E51">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="equal" aboveAverage="0" dxfId="9" text="" percent="0" bottom="0">
@@ -3678,6 +3694,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="AF18"/>
   <autoFilter ref="A1:M26"/>
   <conditionalFormatting sqref="L2:L26">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="10" text="" percent="0" bottom="0">
@@ -3706,13 +3723,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:L28"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="23" min="1" max="1"/>
     <col width="14" customWidth="1" style="23" min="2" max="12"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="31.5" customHeight="1" s="24">
       <c r="B2" s="40" t="inlineStr">
         <is>
@@ -3720,6 +3738,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="21.75" customHeight="1" s="24">
       <c r="B4" s="41" t="inlineStr">
         <is>
@@ -3770,6 +3789,8 @@
       </c>
     </row>
     <row r="6" ht="19.5" customHeight="1" s="24"/>
+    <row r="7"/>
+    <row r="8"/>
     <row r="9" ht="24" customHeight="1" s="24">
       <c r="B9" s="45" t="inlineStr">
         <is>
@@ -4034,6 +4055,7 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="24" customHeight="1" s="24">
       <c r="B22" s="45" t="inlineStr">
         <is>
@@ -4109,6 +4131,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="AF18"/>
   <mergeCells count="13">
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="J4:K4"/>

</xml_diff>